<commit_message>
Align high data center load growth scenario with ADP's high scenario
</commit_message>
<xml_diff>
--- a/InputData/bldgs/BDCL/BAU Data Center Load.xlsx
+++ b/InputData/bldgs/BDCL/BAU Data Center Load.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\bldgs\BDCL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E503E2-C6DE-4C49-96A1-4779AD393C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F0EEEDF-ABB4-4884-A4D1-7846844BA29A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -90,7 +90,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1255" uniqueCount="494">
   <si>
     <t>Year</t>
   </si>
@@ -1571,9 +1571,6 @@
     <t>*Computed Growth Rates Based on BNEF Data Center Report</t>
   </si>
   <si>
-    <t>ADP mid</t>
-  </si>
-  <si>
     <t>Color Code</t>
   </si>
   <si>
@@ -1590,6 +1587,12 @@
   </si>
   <si>
     <t>2030-2050 Demand for Mid and High Scenarios</t>
+  </si>
+  <si>
+    <t>BNEF growth rate</t>
+  </si>
+  <si>
+    <t>ADP mid growth rate</t>
   </si>
 </sst>
 </file>
@@ -1597,7 +1600,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.000%"/>
+    <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1841,7 +1844,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -2304,82 +2307,82 @@
                   <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>240</c:v>
+                  <c:v>279</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>294.66666666666669</c:v>
+                  <c:v>366.79999999998836</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>350.66666666666669</c:v>
+                  <c:v>454.60000000000582</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>410.66666666666669</c:v>
+                  <c:v>542.39999999999418</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>466.66666666666674</c:v>
+                  <c:v>630.19999999998254</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>508.91364902506973</c:v>
+                  <c:v>718</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>554.98521892288238</c:v>
+                  <c:v>783</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>601.05678882069515</c:v>
+                  <c:v>848</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>647.1283587185078</c:v>
+                  <c:v>913</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>693.19992861632045</c:v>
+                  <c:v>978</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>739.2714985141331</c:v>
+                  <c:v>1043</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>764.64630162707408</c:v>
+                  <c:v>1078.7999999999884</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>790.02110474002529</c:v>
+                  <c:v>1114.5999999999913</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>815.39590785297651</c:v>
+                  <c:v>1150.3999999999942</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>840.77071096592772</c:v>
+                  <c:v>1186.1999999999971</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>866.14551407887882</c:v>
+                  <c:v>1222</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>898.53737168396469</c:v>
+                  <c:v>1267.7000000000116</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>930.92922928904011</c:v>
+                  <c:v>1313.4000000000087</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>963.32108689411564</c:v>
+                  <c:v>1359.1000000000058</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>995.71294449919105</c:v>
+                  <c:v>1404.8000000000029</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>1028.1048021042666</c:v>
+                  <c:v>1450.5</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>1060.4966597093523</c:v>
+                  <c:v>1496.2000000000116</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>1092.8885173144279</c:v>
+                  <c:v>1541.9000000000087</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>1125.2803749195034</c:v>
+                  <c:v>1587.6000000000058</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1157.6722325245789</c:v>
+                  <c:v>1633.3000000000029</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>1190.0640901296545</c:v>
+                  <c:v>1679</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3634,32 +3637,32 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
-      <sheetData sheetId="25" refreshError="1"/>
-      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
+      <sheetData sheetId="25"/>
+      <sheetData sheetId="26"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3969,7 +3972,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B8" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -4004,7 +4007,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B17" s="5" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -4025,13 +4028,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B21" s="12" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="E21" s="12"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B23" s="5" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -4419,107 +4422,107 @@
       </c>
       <c r="C2" s="9">
         <f>'Low_Mid_High Scenarios'!C5*10^6</f>
-        <v>240000000</v>
+        <v>279000000</v>
       </c>
       <c r="D2" s="9">
         <f>'Low_Mid_High Scenarios'!D5*10^6</f>
-        <v>294666666.66666669</v>
+        <v>366799999.99998838</v>
       </c>
       <c r="E2" s="9">
         <f>'Low_Mid_High Scenarios'!E5*10^6</f>
-        <v>350666666.66666669</v>
+        <v>454600000.00000584</v>
       </c>
       <c r="F2" s="9">
         <f>'Low_Mid_High Scenarios'!F5*10^6</f>
-        <v>410666666.66666669</v>
+        <v>542399999.99999416</v>
       </c>
       <c r="G2" s="9">
         <f>'Low_Mid_High Scenarios'!G5*10^6</f>
-        <v>466666666.66666675</v>
+        <v>630199999.9999826</v>
       </c>
       <c r="H2" s="9">
         <f>'Low_Mid_High Scenarios'!H5*10^6</f>
-        <v>508913649.02506971</v>
+        <v>718000000</v>
       </c>
       <c r="I2" s="9">
         <f>'Low_Mid_High Scenarios'!I5*10^6</f>
-        <v>554985218.92288244</v>
+        <v>783000000</v>
       </c>
       <c r="J2" s="9">
         <f>'Low_Mid_High Scenarios'!J5*10^6</f>
-        <v>601056788.82069516</v>
+        <v>848000000</v>
       </c>
       <c r="K2" s="9">
         <f>'Low_Mid_High Scenarios'!K5*10^6</f>
-        <v>647128358.71850777</v>
+        <v>913000000</v>
       </c>
       <c r="L2" s="9">
         <f>'Low_Mid_High Scenarios'!L5*10^6</f>
-        <v>693199928.61632049</v>
+        <v>978000000</v>
       </c>
       <c r="M2" s="9">
         <f>'Low_Mid_High Scenarios'!M5*10^6</f>
-        <v>739271498.5141331</v>
+        <v>1043000000</v>
       </c>
       <c r="N2" s="9">
         <f>'Low_Mid_High Scenarios'!N5*10^6</f>
-        <v>764646301.62707412</v>
+        <v>1078799999.9999883</v>
       </c>
       <c r="O2" s="9">
         <f>'Low_Mid_High Scenarios'!O5*10^6</f>
-        <v>790021104.74002528</v>
+        <v>1114599999.9999912</v>
       </c>
       <c r="P2" s="9">
         <f>'Low_Mid_High Scenarios'!P5*10^6</f>
-        <v>815395907.85297656</v>
+        <v>1150399999.9999943</v>
       </c>
       <c r="Q2" s="9">
         <f>'Low_Mid_High Scenarios'!Q5*10^6</f>
-        <v>840770710.96592772</v>
+        <v>1186199999.9999971</v>
       </c>
       <c r="R2" s="9">
         <f>'Low_Mid_High Scenarios'!R5*10^6</f>
-        <v>866145514.07887876</v>
+        <v>1222000000</v>
       </c>
       <c r="S2" s="9">
         <f>'Low_Mid_High Scenarios'!S5*10^6</f>
-        <v>898537371.68396473</v>
+        <v>1267700000.0000117</v>
       </c>
       <c r="T2" s="9">
         <f>'Low_Mid_High Scenarios'!T5*10^6</f>
-        <v>930929229.28904009</v>
+        <v>1313400000.0000088</v>
       </c>
       <c r="U2" s="9">
         <f>'Low_Mid_High Scenarios'!U5*10^6</f>
-        <v>963321086.89411569</v>
+        <v>1359100000.0000057</v>
       </c>
       <c r="V2" s="9">
         <f>'Low_Mid_High Scenarios'!V5*10^6</f>
-        <v>995712944.49919105</v>
+        <v>1404800000.0000029</v>
       </c>
       <c r="W2" s="9">
         <f>'Low_Mid_High Scenarios'!W5*10^6</f>
-        <v>1028104802.1042665</v>
+        <v>1450500000</v>
       </c>
       <c r="X2" s="9">
         <f>'Low_Mid_High Scenarios'!X5*10^6</f>
-        <v>1060496659.7093524</v>
+        <v>1496200000.0000117</v>
       </c>
       <c r="Y2" s="9">
         <f>'Low_Mid_High Scenarios'!Y5*10^6</f>
-        <v>1092888517.3144279</v>
+        <v>1541900000.0000088</v>
       </c>
       <c r="Z2" s="9">
         <f>'Low_Mid_High Scenarios'!Z5*10^6</f>
-        <v>1125280374.9195035</v>
+        <v>1587600000.0000057</v>
       </c>
       <c r="AA2" s="9">
         <f>'Low_Mid_High Scenarios'!AA5*10^6</f>
-        <v>1157672232.524579</v>
+        <v>1633300000.0000029</v>
       </c>
       <c r="AB2" s="9">
         <f>'Low_Mid_High Scenarios'!AB5*10^6</f>
-        <v>1190064090.1296544</v>
+        <v>1679000000</v>
       </c>
     </row>
   </sheetData>
@@ -4890,114 +4893,114 @@
         <f>B3</f>
         <v>200</v>
       </c>
-      <c r="C5" s="29">
-        <f>C4</f>
-        <v>240</v>
-      </c>
-      <c r="D5" s="29">
-        <f t="shared" ref="D5:G5" si="2">D4</f>
-        <v>294.66666666666669</v>
-      </c>
-      <c r="E5" s="29">
+      <c r="C5" s="33">
+        <f>C28</f>
+        <v>279</v>
+      </c>
+      <c r="D5" s="33">
+        <f t="shared" ref="D5:AB5" si="2">D28</f>
+        <v>366.79999999998836</v>
+      </c>
+      <c r="E5" s="33">
         <f t="shared" si="2"/>
-        <v>350.66666666666669</v>
-      </c>
-      <c r="F5" s="29">
+        <v>454.60000000000582</v>
+      </c>
+      <c r="F5" s="33">
         <f t="shared" si="2"/>
-        <v>410.66666666666669</v>
-      </c>
-      <c r="G5" s="29">
+        <v>542.39999999999418</v>
+      </c>
+      <c r="G5" s="33">
         <f t="shared" si="2"/>
-        <v>466.66666666666674</v>
+        <v>630.19999999998254</v>
       </c>
       <c r="H5" s="33">
-        <f t="shared" ref="E5:AB5" si="3">G5*(1+H29)</f>
-        <v>508.91364902506973</v>
+        <f t="shared" si="2"/>
+        <v>718</v>
       </c>
       <c r="I5" s="33">
-        <f t="shared" si="3"/>
-        <v>554.98521892288238</v>
+        <f t="shared" si="2"/>
+        <v>783</v>
       </c>
       <c r="J5" s="33">
-        <f t="shared" si="3"/>
-        <v>601.05678882069515</v>
+        <f t="shared" si="2"/>
+        <v>848</v>
       </c>
       <c r="K5" s="33">
-        <f t="shared" si="3"/>
-        <v>647.1283587185078</v>
+        <f t="shared" si="2"/>
+        <v>913</v>
       </c>
       <c r="L5" s="33">
-        <f t="shared" si="3"/>
-        <v>693.19992861632045</v>
+        <f t="shared" si="2"/>
+        <v>978</v>
       </c>
       <c r="M5" s="33">
-        <f t="shared" si="3"/>
-        <v>739.2714985141331</v>
+        <f t="shared" si="2"/>
+        <v>1043</v>
       </c>
       <c r="N5" s="33">
-        <f t="shared" si="3"/>
-        <v>764.64630162707408</v>
+        <f t="shared" si="2"/>
+        <v>1078.7999999999884</v>
       </c>
       <c r="O5" s="33">
-        <f t="shared" si="3"/>
-        <v>790.02110474002529</v>
+        <f t="shared" si="2"/>
+        <v>1114.5999999999913</v>
       </c>
       <c r="P5" s="33">
-        <f t="shared" si="3"/>
-        <v>815.39590785297651</v>
+        <f t="shared" si="2"/>
+        <v>1150.3999999999942</v>
       </c>
       <c r="Q5" s="33">
-        <f t="shared" si="3"/>
-        <v>840.77071096592772</v>
+        <f t="shared" si="2"/>
+        <v>1186.1999999999971</v>
       </c>
       <c r="R5" s="33">
-        <f t="shared" si="3"/>
-        <v>866.14551407887882</v>
+        <f t="shared" si="2"/>
+        <v>1222</v>
       </c>
       <c r="S5" s="33">
-        <f t="shared" si="3"/>
-        <v>898.53737168396469</v>
+        <f t="shared" si="2"/>
+        <v>1267.7000000000116</v>
       </c>
       <c r="T5" s="33">
-        <f t="shared" si="3"/>
-        <v>930.92922928904011</v>
+        <f t="shared" si="2"/>
+        <v>1313.4000000000087</v>
       </c>
       <c r="U5" s="33">
-        <f t="shared" si="3"/>
-        <v>963.32108689411564</v>
+        <f t="shared" si="2"/>
+        <v>1359.1000000000058</v>
       </c>
       <c r="V5" s="33">
-        <f t="shared" si="3"/>
-        <v>995.71294449919105</v>
+        <f t="shared" si="2"/>
+        <v>1404.8000000000029</v>
       </c>
       <c r="W5" s="33">
-        <f t="shared" si="3"/>
-        <v>1028.1048021042666</v>
+        <f t="shared" si="2"/>
+        <v>1450.5</v>
       </c>
       <c r="X5" s="33">
-        <f t="shared" si="3"/>
-        <v>1060.4966597093523</v>
+        <f t="shared" si="2"/>
+        <v>1496.2000000000116</v>
       </c>
       <c r="Y5" s="33">
-        <f t="shared" si="3"/>
-        <v>1092.8885173144279</v>
+        <f t="shared" si="2"/>
+        <v>1541.9000000000087</v>
       </c>
       <c r="Z5" s="33">
-        <f t="shared" si="3"/>
-        <v>1125.2803749195034</v>
+        <f t="shared" si="2"/>
+        <v>1587.6000000000058</v>
       </c>
       <c r="AA5" s="33">
-        <f t="shared" si="3"/>
-        <v>1157.6722325245789</v>
+        <f t="shared" si="2"/>
+        <v>1633.3000000000029</v>
       </c>
       <c r="AB5" s="33">
-        <f t="shared" si="3"/>
-        <v>1190.0640901296545</v>
+        <f t="shared" si="2"/>
+        <v>1679</v>
       </c>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.35">
@@ -5015,13 +5018,13 @@
     <row r="10" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A10" s="30"/>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>492</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A11" s="31"/>
       <c r="B11" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.35">
@@ -5032,7 +5035,7 @@
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.35">
       <c r="B15" s="4" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.35">
@@ -5144,43 +5147,43 @@
         <v>2030</v>
       </c>
       <c r="I23">
-        <f t="shared" ref="I23:AB23" si="4">H23+1</f>
+        <f t="shared" ref="I23:AB23" si="3">H23+1</f>
         <v>2031</v>
       </c>
       <c r="J23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2032</v>
       </c>
       <c r="K23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2033</v>
       </c>
       <c r="L23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2034</v>
       </c>
       <c r="M23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2035</v>
       </c>
       <c r="N23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2036</v>
       </c>
       <c r="O23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2037</v>
       </c>
       <c r="P23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2038</v>
       </c>
       <c r="Q23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2039</v>
       </c>
       <c r="R23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2040</v>
       </c>
       <c r="S23">
@@ -5188,27 +5191,27 @@
         <v>2041</v>
       </c>
       <c r="T23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2042</v>
       </c>
       <c r="U23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2043</v>
       </c>
       <c r="V23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2044</v>
       </c>
       <c r="W23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2045</v>
       </c>
       <c r="X23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2046</v>
       </c>
       <c r="Y23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2047</v>
       </c>
       <c r="Z23">
@@ -5216,11 +5219,11 @@
         <v>2048</v>
       </c>
       <c r="AA23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2049</v>
       </c>
       <c r="AB23">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2050</v>
       </c>
     </row>
@@ -5341,15 +5344,15 @@
         <v>16</v>
       </c>
       <c r="D25" s="19">
-        <f t="shared" ref="D25:F25" si="5">E25</f>
+        <f t="shared" ref="D25:F25" si="4">E25</f>
         <v>5.6192236598880285E-2</v>
       </c>
       <c r="E25" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>5.6192236598880285E-2</v>
       </c>
       <c r="F25" s="19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>5.6192236598880285E-2</v>
       </c>
       <c r="G25" s="19">
@@ -5369,11 +5372,11 @@
         <v>5.3202660133009783E-2</v>
       </c>
       <c r="K25" s="8">
-        <f t="shared" ref="K25:Y25" si="6">K24/J24-1</f>
+        <f t="shared" ref="K25:Y25" si="5">K24/J24-1</f>
         <v>5.0515121302761257E-2</v>
       </c>
       <c r="L25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>4.8086048718762431E-2</v>
       </c>
       <c r="M25" s="8">
@@ -5381,51 +5384,51 @@
         <v>4.5879867189860368E-2</v>
       </c>
       <c r="N25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2.3953823953832387E-2</v>
       </c>
       <c r="O25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2.3393461104845636E-2</v>
       </c>
       <c r="P25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2.2858716606993124E-2</v>
       </c>
       <c r="Q25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2.2347872913298872E-2</v>
       </c>
       <c r="R25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>2.1859362654725434E-2</v>
       </c>
       <c r="S25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.2113402061857625E-2</v>
       </c>
       <c r="T25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.1968423733126787E-2</v>
       </c>
       <c r="U25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.1826874685457289E-2</v>
       </c>
       <c r="V25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.1688634667994746E-2</v>
       </c>
       <c r="W25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.1553588987214702E-2</v>
       </c>
       <c r="X25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.142162818955228E-2</v>
       </c>
       <c r="Y25" s="8">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>1.1292647765494657E-2</v>
       </c>
       <c r="Z25" s="8">
@@ -5437,7 +5440,7 @@
         <v>1.1043233082708381E-2</v>
       </c>
       <c r="AB25" s="8">
-        <f t="shared" ref="AB25" si="7">AB24/AA24-1</f>
+        <f t="shared" ref="AB25" si="6">AB24/AA24-1</f>
         <v>1.0922612131068821E-2</v>
       </c>
     </row>
@@ -5462,43 +5465,43 @@
         <v>2030</v>
       </c>
       <c r="I27">
-        <f t="shared" ref="I27:R27" si="8">H27+1</f>
+        <f t="shared" ref="I27:R27" si="7">H27+1</f>
         <v>2031</v>
       </c>
       <c r="J27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2032</v>
       </c>
       <c r="K27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2033</v>
       </c>
       <c r="L27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2034</v>
       </c>
       <c r="M27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2035</v>
       </c>
       <c r="N27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2036</v>
       </c>
       <c r="O27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2037</v>
       </c>
       <c r="P27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2038</v>
       </c>
       <c r="Q27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2039</v>
       </c>
       <c r="R27">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>2040</v>
       </c>
       <c r="S27">
@@ -5506,27 +5509,27 @@
         <v>2041</v>
       </c>
       <c r="T27">
-        <f t="shared" ref="T27:Y27" si="9">S27+1</f>
+        <f t="shared" ref="T27:Y27" si="8">S27+1</f>
         <v>2042</v>
       </c>
       <c r="U27">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>2043</v>
       </c>
       <c r="V27">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>2044</v>
       </c>
       <c r="W27">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>2045</v>
       </c>
       <c r="X27">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>2046</v>
       </c>
       <c r="Y27">
-        <f t="shared" si="9"/>
+        <f t="shared" si="8"/>
         <v>2047</v>
       </c>
       <c r="Z27">
@@ -5534,11 +5537,11 @@
         <v>2048</v>
       </c>
       <c r="AA27">
-        <f t="shared" ref="AA27:AB27" si="10">Z27+1</f>
+        <f t="shared" ref="AA27:AB27" si="9">Z27+1</f>
         <v>2049</v>
       </c>
       <c r="AB27">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>2050</v>
       </c>
     </row>
@@ -5663,15 +5666,15 @@
         <v>9.0529247910863475E-2</v>
       </c>
       <c r="D29" s="19">
-        <f t="shared" ref="D29:F29" si="11">E29</f>
+        <f t="shared" ref="D29:F29" si="10">E29</f>
         <v>9.0529247910863475E-2</v>
       </c>
       <c r="E29" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>9.0529247910863475E-2</v>
       </c>
       <c r="F29" s="19">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>9.0529247910863475E-2</v>
       </c>
       <c r="G29" s="19">
@@ -5691,11 +5694,11 @@
         <v>8.3014048531290019E-2</v>
       </c>
       <c r="K29" s="8">
-        <f t="shared" ref="K29:L29" si="12">K28/J28-1</f>
+        <f t="shared" ref="K29:L29" si="11">K28/J28-1</f>
         <v>7.6650943396226356E-2</v>
       </c>
       <c r="L29" s="8">
-        <f t="shared" si="12"/>
+        <f t="shared" si="11"/>
         <v>7.1193866374589243E-2</v>
       </c>
       <c r="M29" s="8">
@@ -5703,51 +5706,51 @@
         <v>6.6462167689161467E-2</v>
       </c>
       <c r="N29" s="8">
-        <f t="shared" ref="N29:Y29" si="13">N28/M28-1</f>
+        <f t="shared" ref="N29:Y29" si="12">N28/M28-1</f>
         <v>3.4324065196537301E-2</v>
       </c>
       <c r="O29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.3185020393032394E-2</v>
       </c>
       <c r="P29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.2119145881933653E-2</v>
       </c>
       <c r="Q29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.1119610570239153E-2</v>
       </c>
       <c r="R29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.018040802563049E-2</v>
       </c>
       <c r="S29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.7397708674314023E-2</v>
       </c>
       <c r="T29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.6049538534350889E-2</v>
       </c>
       <c r="U29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.4795188061517379E-2</v>
       </c>
       <c r="V29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.3625193142518439E-2</v>
       </c>
       <c r="W29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.2531321184508188E-2</v>
       </c>
       <c r="X29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.1506377111348849E-2</v>
       </c>
       <c r="Y29" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>3.0544044913779489E-2</v>
       </c>
       <c r="Z29" s="8">
@@ -5759,7 +5762,7 @@
         <v>2.8785588309395926E-2</v>
       </c>
       <c r="AB29" s="8">
-        <f t="shared" ref="AB29" si="14">AB28/AA28-1</f>
+        <f t="shared" ref="AB29" si="13">AB28/AA28-1</f>
         <v>2.7980162860464786E-2</v>
       </c>
     </row>

</xml_diff>